<commit_message>
Atores do território em grade (gestores e professores) e renumeração da Etapa 3
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/professores_semana2_diagnostico.xlsx
+++ b/kobo/professores_semana2_diagnostico.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J170"/>
+  <dimension ref="A1:J271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2872,221 +2872,276 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>net_actors</t>
+          <t>net_nota</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Atores do território (NET_ACTORS)</t>
+          <t>Atores do território (NET_ACTORS). Existência, contato, parceria e articulação permanente são níveis diferentes — não confunda um com o outro. Só marque "Parceria" ou "Articulação permanente" se a escola já colabora de fato com esse ator; se ele apenas existe no território ou já houve um contato pontual, isso ainda NÃO é parceria.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>net_nota</t>
+          <t>net_rel</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Existência, contato, parceria e articulação permanente são níveis diferentes — não confunda um com o outro. Só marque "Parceria" ou "Articulação permanente" se a escola já colabora de fato com esse ator; se ele apenas existe no território ou já houve um contato pontual, isso ainda NÃO é parceria. Use "Adicionar" para registrar um ator por vez.</t>
+          <t>Q3.11. Para cada tipo de ator, qual é a relação atual da escola com ele?</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>table-list</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>select_one cat_ator</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>net_cat</t>
+          <t>net_rel_01</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Categoria do ator</t>
+          <t>Secretaria de Educação</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>net_nome</t>
+          <t>net_rel_02</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Nome do ator (ex.: UBS Vila Nova)</t>
+          <t>Secretaria de Meio Ambiente</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>select_one sim_nao_nsabe</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>net_existe</t>
+          <t>net_rel_03</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Existe no território?</t>
+          <t>Defesa Civil</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>select_one nivel_rel</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>net_nivel</t>
+          <t>net_rel_04</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Nível de relação</t>
+          <t>Secretaria de Saúde</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>net_contrib_atual</t>
+          <t>net_rel_05</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Contribuições atuais</t>
+          <t>Assistência Social</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>net_contrib_atual_outro</t>
+          <t>net_rel_06</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>selected(${net_contrib_atual}, 'outro')</t>
+          <t>Obras</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>select_multiple contrib</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>net_contrib_pot</t>
+          <t>net_rel_07</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Contribuições potenciais</t>
+          <t>Bombeiros</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>net_contrib_pot_outro</t>
+          <t>net_rel_08</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>selected(${net_contrib_pot}, 'outro')</t>
+          <t>UBS</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>select_one sim_nao</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>net_prioridade</t>
+          <t>net_rel_09</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Prioridade para fortalecimento (NET_PRIORITY_ACTORS) — é um ator prioritário a fortalecer?</t>
+          <t>Vigilância</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>end_repeat</t>
+          <t>select_one nivel_rel_grade</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>net_rel_10</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Outro (poder público)</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>q3_11</t>
+          <t>net_rel_11</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Q3.11. A escola sabe a quem contatar em uma emergência climática?</t>
+          <t>Universidade</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -3098,44 +3153,39 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>q3_12</t>
+          <t>net_rel_12</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Q3.12. Quais são esses contatos?</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>${q3_11}='sim'</t>
-        </is>
-      </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Instituto Federal</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>q3_13</t>
+          <t>net_rel_13</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Q3.13. Existe um procedimento de emergência definido para eventos climáticos?</t>
+          <t>Escola técnica</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -3147,583 +3197,2780 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>q3_14</t>
+          <t>net_rel_14</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Q3.14. Esse procedimento está documentado/formalizado?</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>${q3_13}='sim'</t>
+          <t>Centro de pesquisa</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>q3_15</t>
+          <t>net_rel_15</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Q3.15. Que ações de preparação já foram feitas (simulados, sinalização, etc.)?</t>
-        </is>
-      </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Museu</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>select_multiple canais</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>q3_16</t>
+          <t>net_rel_16</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Q3.16. Canais de comunicação da escola com a comunidade</t>
+          <t>Jardim botânico</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>q3_16_outro</t>
+          <t>net_rel_17</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>selected(${q3_16}, 'outro')</t>
+          <t>Outro (educação/ciência)</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>select_one suficiente</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>q3_17</t>
+          <t>net_rel_18</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Q3.17. Esses canais seriam suficientes numa emergência?</t>
+          <t>Associação de moradores</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>q3_18</t>
+          <t>net_rel_19</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Q3.18. Algum grupo fica de fora desses canais de comunicação?</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>q3_19</t>
+          <t>net_rel_20</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Q3.19. Que capacidades/conhecimentos a comunidade já possui e podem ser mobilizados?</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Ex.: conhecimento tradicional sobre o clima local, organização comunitária, mutirões, saberes de manejo.</t>
-        </is>
-      </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Cooperativa</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>q3_20</t>
+          <t>net_rel_21</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Q3.20. Quais dessas capacidades parecem mais estratégicas de fortalecer?</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Catadores</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>select_multiple barr_artic</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>q3_21</t>
+          <t>net_rel_22</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Q3.21. Barreiras para articular com atores do território</t>
+          <t>Movimentos sociais</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>q3_21_outro</t>
+          <t>net_rel_23</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>selected(${q3_21}, 'outro')</t>
+          <t>Coletivos</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>q3_22</t>
+          <t>net_rel_24</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Q3.22. Descreva um caso concreto de articulação (bem ou malsucedida) com a comunidade/rede</t>
-        </is>
-      </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Grupos culturais</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>q3_23</t>
+          <t>net_rel_25</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Q3.23. Quem participou desse caso?</t>
-        </is>
-      </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>${q3_22} != ''</t>
-        </is>
-      </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Organizações comunitárias/religiosas</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>q3_24</t>
+          <t>net_rel_26</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Q3.24. O que funcionou bem?</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>${q3_22} != ''</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Outro (sociedade civil)</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>q3_25</t>
+          <t>net_rel_27</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Q3.25. Quais foram as dificuldades?</t>
-        </is>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>${q3_22} != ''</t>
-        </is>
-      </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Povos indígenas</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>q3_26</t>
+          <t>net_rel_28</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Q3.26. O que essa experiência ensinou?</t>
-        </is>
-      </c>
-      <c r="F155" t="inlineStr">
-        <is>
-          <t>${q3_22} != ''</t>
-        </is>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Quilombolas</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>q3_27</t>
+          <t>net_rel_29</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Q3.27. Se houvesse uma relação prioritária para fortalecer agora, qual seria?</t>
-        </is>
-      </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Agricultores familiares</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>q3_28</t>
+          <t>net_rel_30</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Q3.28. Por quê?</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>${q3_27} != ''</t>
-        </is>
-      </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Pescadores</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>evid_e3</t>
+          <t>net_rel_31</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Evidências — Evidências sobre participação e redes</t>
+          <t>Comunidades tradicionais</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>evid_e3_nota</t>
+          <t>net_rel_32</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
+          <t>Lideranças</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>select_one tipo_evid</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>evid_e3_tipo</t>
+          <t>net_rel_33</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Tipo de evidência</t>
+          <t>Detentores de conhecimentos locais</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one nivel_rel_grade</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>evid_e3_tipo_outro</t>
+          <t>net_rel_34</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>${evid_e3_tipo}='outro'</t>
+          <t>Outro (comunidades e conhecimentos)</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>evid_e3_desc</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Descreva a evidência</t>
-        </is>
-      </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>end_group</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>evid_e3_anexo</t>
+          <t>net_atual</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Anexo (foto/documento) — opcional</t>
+          <t>Q3.12. Contribuições atuais — o que cada ator parceiro(a) já oferece à escola?</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>(${net_rel_01} = 'parceria' or ${net_rel_01} = 'articulacao') or (${net_rel_02} = 'parceria' or ${net_rel_02} = 'articulacao') or (${net_rel_03} = 'parceria' or ${net_rel_03} = 'articulacao') or (${net_rel_04} = 'parceria' or ${net_rel_04} = 'articulacao') or (${net_rel_05} = 'parceria' or ${net_rel_05} = 'articulacao') or (${net_rel_06} = 'parceria' or ${net_rel_06} = 'articulacao') or (${net_rel_07} = 'parceria' or ${net_rel_07} = 'articulacao') or (${net_rel_08} = 'parceria' or ${net_rel_08} = 'articulacao') or (${net_rel_09} = 'parceria' or ${net_rel_09} = 'articulacao') or (${net_rel_10} = 'parceria' or ${net_rel_10} = 'articulacao') or (${net_rel_11} = 'parceria' or ${net_rel_11} = 'articulacao') or (${net_rel_12} = 'parceria' or ${net_rel_12} = 'articulacao') or (${net_rel_13} = 'parceria' or ${net_rel_13} = 'articulacao') or (${net_rel_14} = 'parceria' or ${net_rel_14} = 'articulacao') or (${net_rel_15} = 'parceria' or ${net_rel_15} = 'articulacao') or (${net_rel_16} = 'parceria' or ${net_rel_16} = 'articulacao') or (${net_rel_17} = 'parceria' or ${net_rel_17} = 'articulacao') or (${net_rel_18} = 'parceria' or ${net_rel_18} = 'articulacao') or (${net_rel_19} = 'parceria' or ${net_rel_19} = 'articulacao') or (${net_rel_20} = 'parceria' or ${net_rel_20} = 'articulacao') or (${net_rel_21} = 'parceria' or ${net_rel_21} = 'articulacao') or (${net_rel_22} = 'parceria' or ${net_rel_22} = 'articulacao') or (${net_rel_23} = 'parceria' or ${net_rel_23} = 'articulacao') or (${net_rel_24} = 'parceria' or ${net_rel_24} = 'articulacao') or (${net_rel_25} = 'parceria' or ${net_rel_25} = 'articulacao') or (${net_rel_26} = 'parceria' or ${net_rel_26} = 'articulacao') or (${net_rel_27} = 'parceria' or ${net_rel_27} = 'articulacao') or (${net_rel_28} = 'parceria' or ${net_rel_28} = 'articulacao') or (${net_rel_29} = 'parceria' or ${net_rel_29} = 'articulacao') or (${net_rel_30} = 'parceria' or ${net_rel_30} = 'articulacao') or (${net_rel_31} = 'parceria' or ${net_rel_31} = 'articulacao') or (${net_rel_32} = 'parceria' or ${net_rel_32} = 'articulacao') or (${net_rel_33} = 'parceria' or ${net_rel_33} = 'articulacao') or (${net_rel_34} = 'parceria' or ${net_rel_34} = 'articulacao')</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>table-list</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>end_repeat</t>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>net_atual_01</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Secretaria de Educação</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>${net_rel_01} = 'parceria' or ${net_rel_01} = 'articulacao'</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>net_atual_02</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Secretaria de Meio Ambiente</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>${net_rel_02} = 'parceria' or ${net_rel_02} = 'articulacao'</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_multiple contrib</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>confirmacao</t>
+          <t>net_atual_03</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Confirmação final</t>
+          <t>Defesa Civil</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>${net_rel_03} = 'parceria' or ${net_rel_03} = 'articulacao'</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_multiple contrib</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>confirmacao_msg</t>
+          <t>net_atual_04</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Semana 2/5 concluída. Obrigado(a) pela sua participação! Suas respostas ajudam a construir um diagnóstico mais completo. Revise o que respondeu, confirme abaixo e clique em Enviar para concluir. ATENÇÃO: depois de clicar em Enviar, aparecerá a mensagem "Submission successful" e o formulário voltará em branco. Isso significa que suas respostas FORAM ENVIADAS. Não preencha nem envie novamente.</t>
+          <t>Secretaria de Saúde</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>${net_rel_04} = 'parceria' or ${net_rel_04} = 'articulacao'</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>select_one confirmo</t>
+          <t>select_multiple contrib</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>confirmacao_envio</t>
+          <t>net_atual_05</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Revisei minhas respostas e confirmo o envio.</t>
-        </is>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>true</t>
+          <t>Assistência Social</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>${net_rel_05} = 'parceria' or ${net_rel_05} = 'articulacao'</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>net_atual_06</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Obras</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>${net_rel_06} = 'parceria' or ${net_rel_06} = 'articulacao'</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>net_atual_07</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Bombeiros</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>${net_rel_07} = 'parceria' or ${net_rel_07} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>net_atual_08</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>${net_rel_08} = 'parceria' or ${net_rel_08} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>net_atual_09</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Vigilância</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>${net_rel_09} = 'parceria' or ${net_rel_09} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>net_atual_10</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Outro (poder público)</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>${net_rel_10} = 'parceria' or ${net_rel_10} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>net_atual_11</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Universidade</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>${net_rel_11} = 'parceria' or ${net_rel_11} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>net_atual_12</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Instituto Federal</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>${net_rel_12} = 'parceria' or ${net_rel_12} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>net_atual_13</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Escola técnica</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>${net_rel_13} = 'parceria' or ${net_rel_13} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>net_atual_14</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Centro de pesquisa</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>${net_rel_14} = 'parceria' or ${net_rel_14} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>net_atual_15</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Museu</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>${net_rel_15} = 'parceria' or ${net_rel_15} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>net_atual_16</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Jardim botânico</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>${net_rel_16} = 'parceria' or ${net_rel_16} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>net_atual_17</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Outro (educação/ciência)</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>${net_rel_17} = 'parceria' or ${net_rel_17} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>net_atual_18</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Associação de moradores</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>${net_rel_18} = 'parceria' or ${net_rel_18} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>net_atual_19</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>${net_rel_19} = 'parceria' or ${net_rel_19} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>net_atual_20</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Cooperativa</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>${net_rel_20} = 'parceria' or ${net_rel_20} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>net_atual_21</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Catadores</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>${net_rel_21} = 'parceria' or ${net_rel_21} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>net_atual_22</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Movimentos sociais</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>${net_rel_22} = 'parceria' or ${net_rel_22} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>net_atual_23</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Coletivos</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>${net_rel_23} = 'parceria' or ${net_rel_23} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>net_atual_24</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Grupos culturais</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>${net_rel_24} = 'parceria' or ${net_rel_24} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>net_atual_25</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Organizações comunitárias/religiosas</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>${net_rel_25} = 'parceria' or ${net_rel_25} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>net_atual_26</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Outro (sociedade civil)</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>${net_rel_26} = 'parceria' or ${net_rel_26} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>net_atual_27</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Povos indígenas</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>${net_rel_27} = 'parceria' or ${net_rel_27} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>net_atual_28</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Quilombolas</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>${net_rel_28} = 'parceria' or ${net_rel_28} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>net_atual_29</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Agricultores familiares</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>${net_rel_29} = 'parceria' or ${net_rel_29} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>net_atual_30</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Pescadores</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>${net_rel_30} = 'parceria' or ${net_rel_30} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>net_atual_31</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Comunidades tradicionais</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>${net_rel_31} = 'parceria' or ${net_rel_31} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>net_atual_32</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Lideranças</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>${net_rel_32} = 'parceria' or ${net_rel_32} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>net_atual_33</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Detentores de conhecimentos locais</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>${net_rel_33} = 'parceria' or ${net_rel_33} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>net_atual_34</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Outro (comunidades e conhecimentos)</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>${net_rel_34} = 'parceria' or ${net_rel_34} = 'articulacao'</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>net_atual_outro</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Especifique (Outro) — contribuições atuais</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>selected(${net_atual_01}, 'outro') or selected(${net_atual_02}, 'outro') or selected(${net_atual_03}, 'outro') or selected(${net_atual_04}, 'outro') or selected(${net_atual_05}, 'outro') or selected(${net_atual_06}, 'outro') or selected(${net_atual_07}, 'outro') or selected(${net_atual_08}, 'outro') or selected(${net_atual_09}, 'outro') or selected(${net_atual_10}, 'outro') or selected(${net_atual_11}, 'outro') or selected(${net_atual_12}, 'outro') or selected(${net_atual_13}, 'outro') or selected(${net_atual_14}, 'outro') or selected(${net_atual_15}, 'outro') or selected(${net_atual_16}, 'outro') or selected(${net_atual_17}, 'outro') or selected(${net_atual_18}, 'outro') or selected(${net_atual_19}, 'outro') or selected(${net_atual_20}, 'outro') or selected(${net_atual_21}, 'outro') or selected(${net_atual_22}, 'outro') or selected(${net_atual_23}, 'outro') or selected(${net_atual_24}, 'outro') or selected(${net_atual_25}, 'outro') or selected(${net_atual_26}, 'outro') or selected(${net_atual_27}, 'outro') or selected(${net_atual_28}, 'outro') or selected(${net_atual_29}, 'outro') or selected(${net_atual_30}, 'outro') or selected(${net_atual_31}, 'outro') or selected(${net_atual_32}, 'outro') or selected(${net_atual_33}, 'outro') or selected(${net_atual_34}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>net_pot</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Q3.13. Contribuições potenciais — o que cada ator que existe no território poderia oferecer?</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>(${net_rel_01} != '' and ${net_rel_01} != 'nao_existe' and ${net_rel_01} != 'nao_sei') or (${net_rel_02} != '' and ${net_rel_02} != 'nao_existe' and ${net_rel_02} != 'nao_sei') or (${net_rel_03} != '' and ${net_rel_03} != 'nao_existe' and ${net_rel_03} != 'nao_sei') or (${net_rel_04} != '' and ${net_rel_04} != 'nao_existe' and ${net_rel_04} != 'nao_sei') or (${net_rel_05} != '' and ${net_rel_05} != 'nao_existe' and ${net_rel_05} != 'nao_sei') or (${net_rel_06} != '' and ${net_rel_06} != 'nao_existe' and ${net_rel_06} != 'nao_sei') or (${net_rel_07} != '' and ${net_rel_07} != 'nao_existe' and ${net_rel_07} != 'nao_sei') or (${net_rel_08} != '' and ${net_rel_08} != 'nao_existe' and ${net_rel_08} != 'nao_sei') or (${net_rel_09} != '' and ${net_rel_09} != 'nao_existe' and ${net_rel_09} != 'nao_sei') or (${net_rel_10} != '' and ${net_rel_10} != 'nao_existe' and ${net_rel_10} != 'nao_sei') or (${net_rel_11} != '' and ${net_rel_11} != 'nao_existe' and ${net_rel_11} != 'nao_sei') or (${net_rel_12} != '' and ${net_rel_12} != 'nao_existe' and ${net_rel_12} != 'nao_sei') or (${net_rel_13} != '' and ${net_rel_13} != 'nao_existe' and ${net_rel_13} != 'nao_sei') or (${net_rel_14} != '' and ${net_rel_14} != 'nao_existe' and ${net_rel_14} != 'nao_sei') or (${net_rel_15} != '' and ${net_rel_15} != 'nao_existe' and ${net_rel_15} != 'nao_sei') or (${net_rel_16} != '' and ${net_rel_16} != 'nao_existe' and ${net_rel_16} != 'nao_sei') or (${net_rel_17} != '' and ${net_rel_17} != 'nao_existe' and ${net_rel_17} != 'nao_sei') or (${net_rel_18} != '' and ${net_rel_18} != 'nao_existe' and ${net_rel_18} != 'nao_sei') or (${net_rel_19} != '' and ${net_rel_19} != 'nao_existe' and ${net_rel_19} != 'nao_sei') or (${net_rel_20} != '' and ${net_rel_20} != 'nao_existe' and ${net_rel_20} != 'nao_sei') or (${net_rel_21} != '' and ${net_rel_21} != 'nao_existe' and ${net_rel_21} != 'nao_sei') or (${net_rel_22} != '' and ${net_rel_22} != 'nao_existe' and ${net_rel_22} != 'nao_sei') or (${net_rel_23} != '' and ${net_rel_23} != 'nao_existe' and ${net_rel_23} != 'nao_sei') or (${net_rel_24} != '' and ${net_rel_24} != 'nao_existe' and ${net_rel_24} != 'nao_sei') or (${net_rel_25} != '' and ${net_rel_25} != 'nao_existe' and ${net_rel_25} != 'nao_sei') or (${net_rel_26} != '' and ${net_rel_26} != 'nao_existe' and ${net_rel_26} != 'nao_sei') or (${net_rel_27} != '' and ${net_rel_27} != 'nao_existe' and ${net_rel_27} != 'nao_sei') or (${net_rel_28} != '' and ${net_rel_28} != 'nao_existe' and ${net_rel_28} != 'nao_sei') or (${net_rel_29} != '' and ${net_rel_29} != 'nao_existe' and ${net_rel_29} != 'nao_sei') or (${net_rel_30} != '' and ${net_rel_30} != 'nao_existe' and ${net_rel_30} != 'nao_sei') or (${net_rel_31} != '' and ${net_rel_31} != 'nao_existe' and ${net_rel_31} != 'nao_sei') or (${net_rel_32} != '' and ${net_rel_32} != 'nao_existe' and ${net_rel_32} != 'nao_sei') or (${net_rel_33} != '' and ${net_rel_33} != 'nao_existe' and ${net_rel_33} != 'nao_sei') or (${net_rel_34} != '' and ${net_rel_34} != 'nao_existe' and ${net_rel_34} != 'nao_sei')</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>table-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>net_pot_01</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Secretaria de Educação</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>${net_rel_01} != '' and ${net_rel_01} != 'nao_existe' and ${net_rel_01} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>net_pot_02</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Secretaria de Meio Ambiente</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>${net_rel_02} != '' and ${net_rel_02} != 'nao_existe' and ${net_rel_02} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>net_pot_03</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Defesa Civil</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>${net_rel_03} != '' and ${net_rel_03} != 'nao_existe' and ${net_rel_03} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>net_pot_04</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Secretaria de Saúde</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>${net_rel_04} != '' and ${net_rel_04} != 'nao_existe' and ${net_rel_04} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>net_pot_05</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Assistência Social</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>${net_rel_05} != '' and ${net_rel_05} != 'nao_existe' and ${net_rel_05} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>net_pot_06</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Obras</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>${net_rel_06} != '' and ${net_rel_06} != 'nao_existe' and ${net_rel_06} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>net_pot_07</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Bombeiros</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>${net_rel_07} != '' and ${net_rel_07} != 'nao_existe' and ${net_rel_07} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>net_pot_08</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>${net_rel_08} != '' and ${net_rel_08} != 'nao_existe' and ${net_rel_08} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>net_pot_09</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Vigilância</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>${net_rel_09} != '' and ${net_rel_09} != 'nao_existe' and ${net_rel_09} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>net_pot_10</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Outro (poder público)</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>${net_rel_10} != '' and ${net_rel_10} != 'nao_existe' and ${net_rel_10} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>net_pot_11</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Universidade</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>${net_rel_11} != '' and ${net_rel_11} != 'nao_existe' and ${net_rel_11} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>net_pot_12</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Instituto Federal</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>${net_rel_12} != '' and ${net_rel_12} != 'nao_existe' and ${net_rel_12} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>net_pot_13</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Escola técnica</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>${net_rel_13} != '' and ${net_rel_13} != 'nao_existe' and ${net_rel_13} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>net_pot_14</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Centro de pesquisa</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>${net_rel_14} != '' and ${net_rel_14} != 'nao_existe' and ${net_rel_14} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>net_pot_15</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Museu</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>${net_rel_15} != '' and ${net_rel_15} != 'nao_existe' and ${net_rel_15} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>net_pot_16</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Jardim botânico</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>${net_rel_16} != '' and ${net_rel_16} != 'nao_existe' and ${net_rel_16} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>net_pot_17</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Outro (educação/ciência)</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>${net_rel_17} != '' and ${net_rel_17} != 'nao_existe' and ${net_rel_17} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>net_pot_18</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Associação de moradores</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>${net_rel_18} != '' and ${net_rel_18} != 'nao_existe' and ${net_rel_18} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>net_pot_19</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>ONG</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>${net_rel_19} != '' and ${net_rel_19} != 'nao_existe' and ${net_rel_19} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>net_pot_20</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Cooperativa</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>${net_rel_20} != '' and ${net_rel_20} != 'nao_existe' and ${net_rel_20} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>net_pot_21</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Catadores</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>${net_rel_21} != '' and ${net_rel_21} != 'nao_existe' and ${net_rel_21} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>net_pot_22</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Movimentos sociais</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>${net_rel_22} != '' and ${net_rel_22} != 'nao_existe' and ${net_rel_22} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>net_pot_23</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Coletivos</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>${net_rel_23} != '' and ${net_rel_23} != 'nao_existe' and ${net_rel_23} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>net_pot_24</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Grupos culturais</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>${net_rel_24} != '' and ${net_rel_24} != 'nao_existe' and ${net_rel_24} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>net_pot_25</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Organizações comunitárias/religiosas</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>${net_rel_25} != '' and ${net_rel_25} != 'nao_existe' and ${net_rel_25} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>net_pot_26</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Outro (sociedade civil)</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>${net_rel_26} != '' and ${net_rel_26} != 'nao_existe' and ${net_rel_26} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>net_pot_27</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Povos indígenas</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>${net_rel_27} != '' and ${net_rel_27} != 'nao_existe' and ${net_rel_27} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>net_pot_28</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Quilombolas</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>${net_rel_28} != '' and ${net_rel_28} != 'nao_existe' and ${net_rel_28} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>net_pot_29</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Agricultores familiares</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>${net_rel_29} != '' and ${net_rel_29} != 'nao_existe' and ${net_rel_29} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>net_pot_30</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Pescadores</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>${net_rel_30} != '' and ${net_rel_30} != 'nao_existe' and ${net_rel_30} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>net_pot_31</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Comunidades tradicionais</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>${net_rel_31} != '' and ${net_rel_31} != 'nao_existe' and ${net_rel_31} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>net_pot_32</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Lideranças</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>${net_rel_32} != '' and ${net_rel_32} != 'nao_existe' and ${net_rel_32} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>net_pot_33</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Detentores de conhecimentos locais</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>${net_rel_33} != '' and ${net_rel_33} != 'nao_existe' and ${net_rel_33} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>select_multiple contrib</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>net_pot_34</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Outro (comunidades e conhecimentos)</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>${net_rel_34} != '' and ${net_rel_34} != 'nao_existe' and ${net_rel_34} != 'nao_sei'</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>net_pot_outro</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Especifique (Outro) — contribuições potenciais</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>selected(${net_pot_01}, 'outro') or selected(${net_pot_02}, 'outro') or selected(${net_pot_03}, 'outro') or selected(${net_pot_04}, 'outro') or selected(${net_pot_05}, 'outro') or selected(${net_pot_06}, 'outro') or selected(${net_pot_07}, 'outro') or selected(${net_pot_08}, 'outro') or selected(${net_pot_09}, 'outro') or selected(${net_pot_10}, 'outro') or selected(${net_pot_11}, 'outro') or selected(${net_pot_12}, 'outro') or selected(${net_pot_13}, 'outro') or selected(${net_pot_14}, 'outro') or selected(${net_pot_15}, 'outro') or selected(${net_pot_16}, 'outro') or selected(${net_pot_17}, 'outro') or selected(${net_pot_18}, 'outro') or selected(${net_pot_19}, 'outro') or selected(${net_pot_20}, 'outro') or selected(${net_pot_21}, 'outro') or selected(${net_pot_22}, 'outro') or selected(${net_pot_23}, 'outro') or selected(${net_pot_24}, 'outro') or selected(${net_pot_25}, 'outro') or selected(${net_pot_26}, 'outro') or selected(${net_pot_27}, 'outro') or selected(${net_pot_28}, 'outro') or selected(${net_pot_29}, 'outro') or selected(${net_pot_30}, 'outro') or selected(${net_pot_31}, 'outro') or selected(${net_pot_32}, 'outro') or selected(${net_pot_33}, 'outro') or selected(${net_pot_34}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>select_multiple cat_ator</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>q3_14</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Q3.14. Quais atores são prioritários para fortalecer a relação? (NET_PRIORITY_ACTORS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>q3_15</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Q3.15. Cite o nome do ator mais relevante para a escola hoje (ex.: UBS Vila Nova)</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>select_one sim_nao_ns</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>q3_16</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Q3.16. A escola sabe a quem contatar em uma emergência climática?</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>q3_17</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Q3.17. Quais são esses contatos?</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>${q3_16}='sim'</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>select_one sim_nao_ns</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>q3_18</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Q3.18. Existe um procedimento de emergência definido para eventos climáticos?</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>select_one sim_nao_ns</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>q3_19</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Q3.19. Esse procedimento está documentado/formalizado?</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>${q3_18}='sim'</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>q3_20</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Q3.20. Que ações de preparação já foram feitas (simulados, sinalização, etc.)?</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>select_multiple canais</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>q3_21</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Q3.21. Canais de comunicação da escola com a comunidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>q3_21_outro</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>selected(${q3_21}, 'outro')</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>select_one suficiente</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>q3_22</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Q3.22. Esses canais seriam suficientes numa emergência?</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>q3_23</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Q3.23. Algum grupo fica de fora desses canais de comunicação?</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>q3_24</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Q3.24. Que capacidades/conhecimentos a comunidade já possui e podem ser mobilizados?</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Ex.: conhecimento tradicional sobre o clima local, organização comunitária, mutirões, saberes de manejo.</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>q3_25</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Q3.25. Quais dessas capacidades parecem mais estratégicas de fortalecer?</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>select_multiple barr_artic</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>q3_26</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Q3.26. Barreiras para articular com atores do território</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>q3_26_outro</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>selected(${q3_26}, 'outro')</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>q3_27</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Q3.27. Descreva um caso concreto de articulação (bem ou malsucedida) com a comunidade/rede</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>q3_28</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Q3.28. Quem participou desse caso?</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>q3_29</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Q3.29. O que funcionou bem?</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>q3_30</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Q3.30. Quais foram as dificuldades?</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>q3_31</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Q3.31. O que essa experiência ensinou?</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>${q3_27} != ''</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>q3_32</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Q3.32. Se houvesse uma relação prioritária para fortalecer agora, qual seria?</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>q3_33</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Q3.33. Por quê?</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>${q3_32} != ''</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>begin_repeat</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>evid_e3</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Evidências — Evidências sobre participação e redes</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>evid_e3_nota</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>select_one tipo_evid</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>evid_e3_tipo</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Tipo de evidência</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>evid_e3_tipo_outro</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>${evid_e3_tipo}='outro'</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>evid_e3_desc</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Descreva a evidência</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>evid_e3_anexo</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Anexo (foto/documento) — opcional</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>end_repeat</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>confirmacao</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Confirmação final</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>confirmacao_msg</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Semana 2/5 concluída. Obrigado(a) pela sua participação! Suas respostas ajudam a construir um diagnóstico mais completo. Revise o que respondeu, confirme abaixo e clique em Enviar para concluir. ATENÇÃO: depois de clicar em Enviar, aparecerá a mensagem "Submission successful" e o formulário voltará em branco. Isso significa que suas respostas FORAM ENVIADAS. Não preencha nem envie novamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>select_one confirmo</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>confirmacao_envio</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Revisei minhas respostas e confirmo o envio.</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>
@@ -3740,7 +5987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C265"/>
+  <dimension ref="A1:C266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7792,85 +10039,85 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>nivel_rel</t>
+          <t>contrib</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>nao_existe</t>
+          <t>recursos</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Não existe relação — não é parceiro(a)</t>
+          <t>Recursos</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>nivel_rel</t>
+          <t>contrib</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>sabe_existe</t>
+          <t>formacao</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Sabe que existe, mas nunca houve contato — não é parceiro(a)</t>
+          <t>Formação</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>nivel_rel</t>
+          <t>contrib</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>contato_pontual</t>
+          <t>articulacao_institucional</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Já houve contato pontual, sem combinação formal — ainda não é parceiro(a)</t>
+          <t>Articulação institucional</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>nivel_rel</t>
+          <t>contrib</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>parceria</t>
+          <t>apoio_tecnico</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Parceria — já colaboram em ações combinadas</t>
+          <t>Apoio técnico</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>nivel_rel</t>
+          <t>contrib</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>articulacao</t>
+          <t>mobilizacao_comunitaria</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Articulação permanente — parceria contínua e estruturada</t>
+          <t>Mobilização comunitária</t>
         </is>
       </c>
     </row>
@@ -7882,12 +10129,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>recursos</t>
+          <t>conhecimentos_tradicionais_locai</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Recursos</t>
+          <t>Conhecimentos tradicionais/locais</t>
         </is>
       </c>
     </row>
@@ -7899,97 +10146,97 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>formacao</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Formação</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>articulacao_institucional</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Articulação institucional</t>
+          <t>WhatsApp</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>apoio_tecnico</t>
+          <t>comunicados_impressos</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Apoio técnico</t>
+          <t>Comunicados impressos</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>mobilizacao_comunitaria</t>
+          <t>reunioes</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Mobilização comunitária</t>
+          <t>Reuniões</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>conhecimentos_tradicionais_locai</t>
+          <t>redes_sociais</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Conhecimentos tradicionais/locais</t>
+          <t>Redes sociais</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>contrib</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>alto_falante_radio_local</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Alto-falante/rádio local</t>
         </is>
       </c>
     </row>
@@ -8001,250 +10248,267 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>comunicados_impressos</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Comunicados impressos</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>reunioes</t>
+          <t>parcialmente</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Reuniões</t>
+          <t>Parcialmente</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>redes_sociais</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Redes sociais</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>alto_falante_radio_local</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Alto-falante/rádio local</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>falta_de_contato</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Falta de contato</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>burocracia</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Burocracia</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>parcialmente</t>
+          <t>desconfianca_historico_de_relaca</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Parcialmente</t>
+          <t>Desconfiança/histórico de relação</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>falta_de_tempo</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Falta de tempo</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>falta_de_contato</t>
+          <t>nao_existe</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Falta de contato</t>
+          <t>Não existe no território</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>burocracia</t>
+          <t>nao_sei</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Burocracia</t>
+          <t>Não sei se existe</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>desconfianca_historico_de_relaca</t>
+          <t>sem_contato</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Desconfiança/histórico de relação</t>
+          <t>Existe, mas nunca houve contato</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>falta_de_tempo</t>
+          <t>contato_pontual</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Falta de tempo</t>
+          <t>Contato pontual, sem combinação formal (ainda não é parceiro(a))</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>parceria</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Parceria — já colaboram em ações combinadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>nivel_rel_grade</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>articulacao</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Articulação permanente — parceria contínua e estruturada</t>
         </is>
       </c>
     </row>

</xml_diff>